<commit_message>
feat: agregar info geografica y actualizar matricula 2026
</commit_message>
<xml_diff>
--- a/data/Fuentes de datos/Reporte de matrícula/01_Matricula_2026.xlsx
+++ b/data/Fuentes de datos/Reporte de matrícula/01_Matricula_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eduardoavendano/Desktop/Datos Mapa Landing/Trabajo Fernando/reportes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jorge\Documents\GOBIERNO_DE_DATOS\Data_Steward\Observatorio_de_Educación\data\Fuentes de datos\Reporte de matrícula\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39039CE4-A99D-984B-BF12-967E0106B1E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B6A506A-E440-466D-929A-F38DBE0905C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16660" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Por sector" sheetId="1" r:id="rId1"/>
@@ -639,9 +639,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -649,7 +652,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -657,7 +660,7 @@
         <v>143747</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -665,7 +668,7 @@
         <v>159469</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -673,7 +676,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -689,9 +692,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -708,7 +715,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -725,7 +732,7 @@
         <v>7160</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -742,7 +749,7 @@
         <v>17409</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -759,7 +766,7 @@
         <v>124324</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -776,7 +783,7 @@
         <v>98998</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -793,7 +800,7 @@
         <v>40095</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -810,7 +817,7 @@
         <v>976</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -827,7 +834,7 @@
         <v>15043</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -844,7 +851,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -869,9 +876,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -888,7 +901,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -905,7 +918,7 @@
         <v>6087</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -922,7 +935,7 @@
         <v>8101</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -939,7 +952,7 @@
         <v>5435</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -956,7 +969,7 @@
         <v>11541</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -973,7 +986,7 @@
         <v>8740</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -990,7 +1003,7 @@
         <v>14652</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1007,7 +1020,7 @@
         <v>11184</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1024,7 +1037,7 @@
         <v>13204</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -1041,7 +1054,7 @@
         <v>6561</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1058,7 +1071,7 @@
         <v>11520</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>26</v>
       </c>
@@ -1075,7 +1088,7 @@
         <v>13788</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>27</v>
       </c>
@@ -1092,7 +1105,7 @@
         <v>8846</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>28</v>
       </c>
@@ -1109,7 +1122,7 @@
         <v>22107</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -1126,7 +1139,7 @@
         <v>25902</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -1143,7 +1156,7 @@
         <v>18479</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>31</v>
       </c>
@@ -1160,7 +1173,7 @@
         <v>14336</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -1177,7 +1190,7 @@
         <v>5422</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>33</v>
       </c>
@@ -1194,7 +1207,7 @@
         <v>18061</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>34</v>
       </c>
@@ -1211,7 +1224,7 @@
         <v>17274</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>35</v>
       </c>
@@ -1228,7 +1241,7 @@
         <v>5313</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>36</v>
       </c>
@@ -1245,7 +1258,7 @@
         <v>23489</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>37</v>
       </c>
@@ -1262,7 +1275,7 @@
         <v>18861</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>38</v>
       </c>
@@ -1279,7 +1292,7 @@
         <v>3171</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>39</v>
       </c>
@@ -1296,7 +1309,7 @@
         <v>827</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>40</v>
       </c>
@@ -1313,7 +1326,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>41</v>
       </c>
@@ -1330,7 +1343,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>42</v>
       </c>
@@ -1347,7 +1360,7 @@
         <v>3847</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>43</v>
       </c>
@@ -1364,7 +1377,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>44</v>
       </c>
@@ -1381,7 +1394,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>45</v>
       </c>
@@ -1398,7 +1411,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>46</v>
       </c>
@@ -1415,7 +1428,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>47</v>
       </c>
@@ -1432,7 +1445,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>48</v>
       </c>
@@ -1449,7 +1462,7 @@
         <v>1182</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>49</v>
       </c>
@@ -1466,7 +1479,7 @@
         <v>2276</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>50</v>
       </c>
@@ -1483,7 +1496,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>51</v>
       </c>
@@ -1500,7 +1513,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>52</v>
       </c>
@@ -1517,7 +1530,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>53</v>
       </c>
@@ -1534,7 +1547,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>5</v>
       </c>
@@ -1559,9 +1572,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>54</v>
       </c>
@@ -1578,7 +1591,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>55</v>
       </c>
@@ -1595,7 +1608,7 @@
         <v>151345</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>56</v>
       </c>
@@ -1612,7 +1625,7 @@
         <v>152946</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1637,9 +1650,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:BC43"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -1704,7 +1717,7 @@
       <c r="BB1" s="1"/>
       <c r="BC1" s="1"/>
     </row>
-    <row r="2" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>58</v>
       </c>
@@ -1817,7 +1830,7 @@
       </c>
       <c r="BC2" s="1"/>
     </row>
-    <row r="3" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>64</v>
       </c>
@@ -1984,12 +1997,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2156,7 +2169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -2323,7 +2336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -2490,7 +2503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -2657,7 +2670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -2824,7 +2837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -2991,7 +3004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -3158,7 +3171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -3325,7 +3338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -3492,7 +3505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -3659,7 +3672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -3826,7 +3839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>27</v>
       </c>
@@ -3993,7 +4006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>28</v>
       </c>
@@ -4160,7 +4173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>29</v>
       </c>
@@ -4327,7 +4340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>30</v>
       </c>
@@ -4494,7 +4507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>31</v>
       </c>
@@ -4661,7 +4674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -4828,7 +4841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>33</v>
       </c>
@@ -4995,7 +5008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>34</v>
       </c>
@@ -5162,7 +5175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>35</v>
       </c>
@@ -5329,7 +5342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>36</v>
       </c>
@@ -5496,7 +5509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>37</v>
       </c>
@@ -5663,7 +5676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>38</v>
       </c>
@@ -5830,7 +5843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>39</v>
       </c>
@@ -5997,7 +6010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -6164,7 +6177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>41</v>
       </c>
@@ -6331,7 +6344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>42</v>
       </c>
@@ -6498,7 +6511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>43</v>
       </c>
@@ -6665,7 +6678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>44</v>
       </c>
@@ -6832,7 +6845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>45</v>
       </c>
@@ -6999,7 +7012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>46</v>
       </c>
@@ -7166,7 +7179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>47</v>
       </c>
@@ -7333,7 +7346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>48</v>
       </c>
@@ -7500,7 +7513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>49</v>
       </c>
@@ -7667,7 +7680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>50</v>
       </c>
@@ -7834,7 +7847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>51</v>
       </c>
@@ -8001,7 +8014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>52</v>
       </c>
@@ -8168,7 +8181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>53</v>
       </c>
@@ -8335,7 +8348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:55" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>65</v>
       </c>
@@ -8504,6 +8517,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="AV2:AW2"/>
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="AJ2:AK2"/>
+    <mergeCell ref="AL2:AM2"/>
+    <mergeCell ref="AR2:AS2"/>
+    <mergeCell ref="AT2:AU2"/>
+    <mergeCell ref="B1:S1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="N2:O2"/>
     <mergeCell ref="AZ2:BA2"/>
     <mergeCell ref="BB2:BC2"/>
     <mergeCell ref="AX2:AY2"/>
@@ -8520,20 +8547,6 @@
     <mergeCell ref="AP2:AQ2"/>
     <mergeCell ref="AH2:AI2"/>
     <mergeCell ref="J2:K2"/>
-    <mergeCell ref="AR2:AS2"/>
-    <mergeCell ref="AT2:AU2"/>
-    <mergeCell ref="B1:S1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="AV2:AW2"/>
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="R2:S2"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="AJ2:AK2"/>
-    <mergeCell ref="AL2:AM2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8542,132 +8555,132 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:A30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="61.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="61.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>89</v>
       </c>

</xml_diff>

<commit_message>
docs: agregar reporte de diferencias entre data historica 2020-2025 y data 2026
</commit_message>
<xml_diff>
--- a/data/Fuentes de datos/Reporte de matrícula/01_Matricula_2026.xlsx
+++ b/data/Fuentes de datos/Reporte de matrícula/01_Matricula_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jorge\Documents\GOBIERNO_DE_DATOS\Data_Steward\Observatorio_de_Educación\data\Fuentes de datos\Reporte de matrícula\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B6A506A-E440-466D-929A-F38DBE0905C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F1C0DA1-E246-4546-813F-12521124C033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Por sector" sheetId="1" r:id="rId1"/>
@@ -8517,21 +8517,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="AV2:AW2"/>
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="R2:S2"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="AJ2:AK2"/>
-    <mergeCell ref="AL2:AM2"/>
-    <mergeCell ref="AR2:AS2"/>
-    <mergeCell ref="AT2:AU2"/>
-    <mergeCell ref="B1:S1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="AZ2:BA2"/>
     <mergeCell ref="BB2:BC2"/>
     <mergeCell ref="AX2:AY2"/>
     <mergeCell ref="T1:AK1"/>
@@ -8547,6 +8532,21 @@
     <mergeCell ref="AP2:AQ2"/>
     <mergeCell ref="AH2:AI2"/>
     <mergeCell ref="J2:K2"/>
+    <mergeCell ref="B1:S1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="AZ2:BA2"/>
+    <mergeCell ref="AV2:AW2"/>
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="AJ2:AK2"/>
+    <mergeCell ref="AL2:AM2"/>
+    <mergeCell ref="AR2:AS2"/>
+    <mergeCell ref="AT2:AU2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>